<commit_message>
Update scholarships, career opportunities and magazine extraction (29 Oct 2026)
</commit_message>
<xml_diff>
--- a/career-magazines/PratiyogitaDarpan_Log_Apr2025-Sep2026.xlsx
+++ b/career-magazines/PratiyogitaDarpan_Log_Apr2025-Sep2026.xlsx
@@ -692,7 +692,7 @@
     <row r="4" ht="15" customHeight="1" s="17">
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>Compiled 28 October 2026 | updated 28 October 2026 with the 21-28 October 2026 scrape</t>
+          <t>Compiled 28 October 2026 | updated 29 October 2026 with the November 2026 issue admissions/entrance entries (CLAT 2027, UGC NET Dec 2026, CSIR-UGC NET Dec 2026, NIFTEE 2027, NMAT 2026-27)</t>
         </is>
       </c>
     </row>
@@ -824,8 +824,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B11:D12"/>
     <mergeCell ref="B9:D10"/>
-    <mergeCell ref="B11:D12"/>
     <mergeCell ref="B7:D8"/>
     <mergeCell ref="B13:D14"/>
   </mergeCells>
@@ -841,7 +841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="16" min="1" max="1"/>
@@ -2877,6 +2877,431 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Admission / Entrance Exam</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CLAT 2027 (Common Law Admission Test)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Consortium of National Law Universities</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Class 12 / Intermediate students and above seeking admission to 5-year integrated law programmes at NLUs</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>All categories</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Boys and girls</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>As per CLAT 2027 rules</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Annual (2027 intake)</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Application fee as notified; no scholarship advertised in the notice</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Applications open till 31-Oct-2026; exam 06-Dec-2026</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Open now - closes 31-Oct-2026</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>https://consortiumofnlus.ac.in</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>consortiumofnlus.ac.in; pratiyogitakosh.com admission notices (posted 05-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Dates verified on the official exam portal; appearance in the November 2026 issue is inferred from Pratiyogita Darpan's standard admissions/entrance coverage and is not page-verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Admission / Entrance Exam</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>UGC NET December 2026</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>National Testing Agency (NTA) for UGC</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>PG degree holders (or equivalent) seeking eligibility for Assistant Professor and Junior Research Fellowship</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>All categories</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Boys and girls</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>No upper age limit for Assistant Professor; JRF as per UGC rules</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Twice a year (June and December sessions)</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Application fee as notified; JRF carries a monthly fellowship</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Revised bulletin: application last date 31-Oct-2026 with late fee; correction window 02-04 Nov 2026; exam 14-21 Dec 2026</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Open now - late-fee window closes 31-Oct-2026</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>https://ugcnet.nta.ac.in</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>ugcnet.nta.ac.in; pratiyogitakosh.com admission notices (posted 16-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Dates verified on the official exam portal; appearance in the November 2026 issue is inferred from Pratiyogita Darpan's standard admissions/entrance coverage and is not page-verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Admission / Entrance Exam</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Joint CSIR-UGC NET December 2026</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>National Testing Agency (NTA) for CSIR</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>M.Sc / BE / B.Tech / B.Pharma / MBBS and equivalent science graduates for PhD admission and JRF-Lectureship</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>All categories</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Boys and girls</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>JRF as per CSIR rules; Lectureship no upper limit</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Twice a year (June and December sessions)</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Application fee as notified; JRF/SRF carry monthly fellowship</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Apply 07-Oct-2026 to 05-Nov-2026; exam 19, 22 and 27-Dec-2026</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Open now - apply by 05-Nov-2026</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>https://csirnet.nta.ac.in</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>csirnet.nta.ac.in; pratiyogitakosh.com admission notices (posted 07-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Dates verified on the official exam portal; appearance in the November 2026 issue is inferred from Pratiyogita Darpan's standard admissions/entrance coverage and is not page-verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Admission / Entrance Exam</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>NIFT Entrance Examination (NIFTEE) 2027</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>National Institute of Fashion Technology (NIFT), exam conducted by NTA</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Class 12 / Intermediate for B.Des and B.FTech; graduation for M.Des, M.FTech and MFM</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>All categories</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Boys and girls</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>As per NIFT 2027 rules (upper limit relaxed for reserved categories)</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Annual (2027 intake)</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Application fee as notified; fee-based programmes</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Apply by 16-Nov-2026; exam 10-Jan-2027</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Open now - apply by 16-Nov-2026</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>https://nift.nta.nic.in</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>nift.nta.nic.in; pratiyogitakosh.com admission notices (posted 18-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Dates verified on the official exam portal; appearance in the November 2026 issue is inferred from Pratiyogita Darpan's standard admissions/entrance coverage and is not page-verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Admission / Entrance Exam</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>NMAT by GMAC 2026-27 (NMIMS / GMAC management admission test)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Graduate Management Admission Council (GMAC)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Graduates seeking admission to MBA / PGDM programmes that accept NMAT scores</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>All categories</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Boys and girls</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>As per NMAT 2026-27 rules</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Annual (2026-27 admission cycle)</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Application fee as notified; retake options available</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Registration closed; exam window opens 02-Nov-2026</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Upcoming - exam window from 02-Nov-2026</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>https://www.mba.com/exams/nmat</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>mba.com; pratiyogitakosh.com admission notices (posted 25-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Dates verified on the official exam portal; appearance in the November 2026 issue is inferred from Pratiyogita Darpan's standard admissions/entrance coverage and is not page-verified.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q20"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>